<commit_message>
docs: finalize monochrome context diagram, preview and excel script
</commit_message>
<xml_diff>
--- a/docs/FA26SE032_GFA96_MinhTTH5.xlsx
+++ b/docs/FA26SE032_GFA96_MinhTTH5.xlsx
@@ -925,22 +925,22 @@
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="14" customWidth="1" style="45" min="1" max="1"/>
-    <col width="42" customWidth="1" style="45" min="2" max="2"/>
+    <col width="44" customWidth="1" style="45" min="2" max="2"/>
     <col width="24" customWidth="1" style="45" min="3" max="3"/>
     <col width="38" customWidth="1" style="45" min="4" max="12"/>
-    <col width="38" customWidth="1" style="45" min="5" max="5"/>
-    <col width="42" customWidth="1" style="45" min="6" max="6"/>
-    <col width="32" customWidth="1" style="45" min="7" max="7"/>
-    <col width="32" customWidth="1" style="45" min="8" max="8"/>
-    <col width="32" customWidth="1" style="45" min="9" max="9"/>
-    <col width="32" customWidth="1" style="45" min="10" max="10"/>
-    <col width="32" customWidth="1" style="45" min="11" max="11"/>
-    <col width="32" customWidth="1" style="45" min="12" max="12"/>
-    <col width="32" customWidth="1" style="45" min="13" max="17"/>
-    <col width="32" customWidth="1" style="45" min="14" max="14"/>
-    <col width="32" customWidth="1" style="45" min="15" max="15"/>
-    <col width="32" customWidth="1" style="45" min="16" max="16"/>
-    <col width="32" customWidth="1" style="45" min="17" max="17"/>
+    <col width="40" customWidth="1" style="45" min="5" max="5"/>
+    <col width="44" customWidth="1" style="45" min="6" max="6"/>
+    <col width="46" customWidth="1" style="45" min="7" max="7"/>
+    <col width="34" customWidth="1" style="45" min="8" max="8"/>
+    <col width="34" customWidth="1" style="45" min="9" max="9"/>
+    <col width="34" customWidth="1" style="45" min="10" max="10"/>
+    <col width="34" customWidth="1" style="45" min="11" max="11"/>
+    <col width="34" customWidth="1" style="45" min="12" max="12"/>
+    <col width="34" customWidth="1" style="45" min="13" max="17"/>
+    <col width="34" customWidth="1" style="45" min="14" max="14"/>
+    <col width="34" customWidth="1" style="45" min="15" max="15"/>
+    <col width="34" customWidth="1" style="45" min="16" max="16"/>
+    <col width="34" customWidth="1" style="45" min="17" max="17"/>
     <col width="8.77734375" customWidth="1" style="45" min="18" max="27"/>
   </cols>
   <sheetData>
@@ -1174,7 +1174,7 @@
       <c r="Z5" s="56" t="n"/>
       <c r="AA5" s="44" t="n"/>
     </row>
-    <row r="6" ht="290" customHeight="1" s="45">
+    <row r="6" ht="360" customHeight="1" s="45">
       <c r="A6" s="71" t="inlineStr">
         <is>
           <t>FA26SE032</t>
@@ -1196,114 +1196,125 @@
         <is>
           <t>✅ [HOÀN THÀNH 100%]
 • Phê duyệt KH chi tiết thực hiện khóa luận, supervisor phê duyệt.
-• Thiết kế kiến trúc SAD, đặc tả SRS, tài liệu bảo mật Gitignore.
-• Thiết kế CSDL Master 21 bảng 3NF (PostgreSQL) &amp; kịch bản gieo mầm seed data.
+• Thiết kế kiến trúc tổng thể phần mềm SAD, đặc tả yêu cầu chức năng SRS.
+• Thiết kế CSDL Master 41 bảng chuẩn 3NF (PostgreSQL) &amp; kịch bản gieo mầm dữ liệu mẫu.
 • Khởi tạo Base Monorepo NestJS + React Vite + Docker Multi-Container.</t>
         </is>
       </c>
       <c r="E6" s="74" t="inlineStr">
         <is>
           <t>✅ [HOÀN THÀNH 100%]
-• Hoàn thiện FR-01 → FR-08 (IAM, Bảo mật Argon2id/JWT/Bcrypt/OTP, Quản lý Gian hàng, Sản phẩm &amp; Media Hub).
-• Hoàn thiện FR-09 → FR-16 (Dynamic Smart Link, Dynamic QR Code canvas 512x512, Last-Click Cookie 30 ngày, Redis Sliding Window chống click tặc, Đặt hàng khách vãng lai).
-• Hoàn thiện FR-31 &amp; FR-32 (AI Fraud Sentinel phát hiện gian lận traffic, Hệ thống Audit Logs an ninh bất biến 16/16 test suites pass).</t>
+• Phân hệ Quản trị &amp; Xác thực tài khoản: Đăng ký/đăng nhập đa vai trò, bảo mật mật khẩu Argon2id, mã JWT, xác thực 2 bước (2FA OTP), Quản lý Gian hàng đối tác, Danh mục Sản phẩm &amp; Kho nội dung số quảng bá.
+• Phân hệ Tiếp thị liên kết (Affiliate Tracking): Tự động tạo Link tiếp thị rút gọn, tạo mã QR Code động canvas 512x512, cơ chế lưu Cookie người mua 30 ngày, thuật toán chặn click ảo/spam bằng Redis.
+• Khởi tạo Cổng Khách Hàng (Customer Portal) &amp; Sổ địa chỉ giao nhận.
+• Thiết lập chuỗi an ninh kiểm toán Audit Logs bất biến SHA-256 (16/16 kịch bản kiểm thử đạt chuẩn).</t>
         </is>
       </c>
-      <c r="F6" s="75" t="inlineStr">
+      <c r="F6" s="74" t="inlineStr">
         <is>
-          <t>⭐ [ĐANG BÁO CÁO - HOÀN THÀNH XUẤT SẮC 100%]
-1. Phân hệ Tài chính, Đơn hàng &amp; Hoa hồng (FR-17 → FR-24):
-   - Xử lý đơn hàng đa trạng thái, cơ chế Escrow 14 ngày bảo đảm chính sách đổi trả.
-   - Tự động quyết toán hoa hồng vào số dư ví CTV sau 14 ngày (0đ phí ngân hàng nhờ hạch toán sổ cái nội bộ).
+          <t>✅ [HOÀN THÀNH 100%]
+1. Phân hệ Tài chính, Đơn hàng &amp; Quyết toán hoa hồng:
+   - Xử lý đơn hàng đa trạng thái; nền tảng Quỹ bảo chứng Escrow 14 ngày bảo đảm quyền lợi đổi trả.
+   - Tự động quyết toán hoa hồng vào ví CTV nội bộ (0đ phí ngân hàng nhờ hạch toán sổ cái kép).
    - Khấu trừ thuế TNCN 10% theo luật với lệnh thanh toán &gt;= 2 triệu VNĐ.
    - Tạo quy trình giải ngân hàng loạt Batch Payout theo file VietQR Napas247 XLSX.
-2. Phân tách chuẩn hóa 5 vai trò hệ thống:
-   - Tách rời riêng biệt SYSTEM_MANAGER (Vận hành &amp; Tuân thủ: duyệt KYC CCCD/MST, tranh chấp) và SYSTEM_ADMIN (Quản trị tối cao: phân quyền RBAC, an ninh sàn).
+2. Phân tách chuẩn hóa vai trò hệ thống:
+   - Tách biệt rõ ràng SYSTEM_MANAGER (vận hành thẩm định KYC CCCD/MST, kiểm duyệt sản phẩm) và SYSTEM_ADMIN (quản trị tối cao, phân quyền RBAC, an ninh sàn).
 3. Chuẩn hóa Design System Vàng Be (Warm Sand Gold):
-   - Tái thiết kế trang Đăng nhập (/login) sang trọng, duyên dáng, tích hợp bộ kiểm thử 5 vai trò mượt mà không bị cắt chữ.
-   - Đồng bộ Public Header, Search Zoom Modal và Marketplace Shopee-style.
-4. Kiểm thử &amp; Git:
-   - Kéo code mới từ origin/main hợp nhất 0 conflict (Merge PR #50, #51).
-   - Build Frontend (1.01s) &amp; Backend 0 lỗi; Push code an toàn lên branch thang.</t>
+   - Tái thiết kế trang Login (/login) sang trọng, tích hợp bộ chuyển đổi 5 vai trò mượt mà.
+   - Đồng bộ Public Header, Search Zoom Modal và Marketplace Shopee-style; Sơ đồ Use Case Bill OTP (PR #50, #51).
+4. Tái cấu trúc phân công 4 thành viên độc lập, chuẩn hóa luồng nghiệp vụ E-commerce thực tế.</t>
         </is>
       </c>
-      <c r="G6" s="76" t="inlineStr">
+      <c r="G6" s="75" t="inlineStr">
         <is>
-          <t>⏳ [KẾ HOẠCH DỰ KIẾN]
-• Hoàn thiện FR-25 → FR-30:
-  - Socket.io Chat realtime đa kênh giữa KOL và Chủ Gian hàng.
-  - Quy trình gửi &amp; duyệt mẫu thử sản phẩm (Sample Request).
-  - Động cơ AI Gợi ý KOL phù hợp với từng danh mục sản phẩm của Shop.</t>
+          <t>⭐ [ĐANG BÁO CÁO - HOÀN THÀNH 100%]
+1. Phân hệ Bảo Mật, Escrow &amp; IAM:
+   - Khóa 100% bắt buộc đăng nhập (Google 1-Click 1.5s), Quên mật khẩu OTP Email 5 phút, mã hóa Argon2id.
+   - Quỹ Escrow 14 ngày thích ứng nghỉ Lễ/Tết VN, Cổng Trọng tài phân xử tranh chấp đổi trả (Split-View).
+   - Trung tâm thông báo toàn sàn thời gian thực đa vai trò &amp; Động cơ AI Fraud Sentinel chống tự mua.
+2. Phân hệ Quản Trị Gian Hàng &amp; Vận Chuyển:
+   - Quản lý tồn kho tức thời (cảnh báo &lt;= 5 sp), Shop chủ động hủy đơn có lý do kèm tự hoàn tiền ví khách.
+   - Shipping Simulator in phiếu giao hàng A6 có mã vạch Barcode, Thẩm định video đổi trả 14 ngày &amp; Voucher riêng.
+3. Phân hệ Mạng Lưới KOL/KOC &amp; Quản Trị Sàn:
+   - Phân cấp hoa hồng 2 tầng (công khai &amp; deal riêng), Quy trình xin mẫu thử 4 bước (cam kết trả video 14 ngày).
+   - Voucher Livestream phiên live có đồng hồ đếm ngược tự hủy, Hàng đợi duyệt hồ sơ Shop &amp; Duyệt sản phẩm.
+4. Phân hệ Cổng Khách Hàng:
+   - Giỏ hàng đồng bộ Database PostgreSQL đa thiết bị, Quy trình gửi khiếu nại đổi trả 14 ngày (bắt buộc video mở hộp).
+   - Ràng buộc đánh giá thật Verified Review Gate (chỉ đơn COMPLETED), Minh bạch chính sách bảo hành &amp; Chat Khách ⇄ Shop.
+5. Công tác Chuẩn bị Báo cáo &amp; Review Tiến Độ với GVHD:
+   - Đóng gói kịch bản Demo hoàn chỉnh luồng nghiệp vụ E2E: Mua hàng -&gt; Giao vận -&gt; Escrow bảo chứng -&gt; Đổi trả/Hoàn tất.
+   - Hoàn thiện Slide báo cáo tiến độ, cập nhật tài liệu kiến trúc SAD, sơ đồ Use Case và rà soát hệ thống sẵn sàng phản biện.</t>
         </is>
       </c>
       <c r="H6" s="76" t="inlineStr">
         <is>
           <t>⏳ [KẾ HOẠCH DỰ KIẾN]
-• Hoàn thiện Bảng vinh danh Top KOL (Leaderboard Gamification).
-• Báo cáo tài chính &amp; Biểu đồ Doanh số Realtime qua Recharts.
-• Phân tích phễu chuyển đổi (Traffic -&gt; Click -&gt; Lead -&gt; Order -&gt; Paid).</t>
+• Hoàn thiện Socket.io In-App Chat Realtime đa kênh: Khách hàng ⇄ Chủ Shop (tư vấn sản phẩm) và KOL ⇄ Chủ Shop (đàm phán deal hoa hồng độc quyền Exclusive Deal).
+• Tích hợp Voucher Livestream có đếm ngược thời gian thực vào giao diện phiên phát sóng; tối ưu cơ chế tự hủy voucher khi hết phiên.</t>
         </is>
       </c>
       <c r="I6" s="76" t="inlineStr">
         <is>
           <t>⏳ [KẾ HOẠCH DỰ KIẾN]
-• Kiểm thử tích hợp hệ thống toàn diện E2E (End-to-End Testing) bao phủ toàn bộ 32 yêu cầu chức năng (FR-01 → FR-32).
-• Tối ưu hóa phản hồi API qua Postman/Newman automation test.</t>
+• Xây dựng Bảng vinh danh Top KOL (Leaderboard Gamification) thúc đẩy cạnh tranh doanh số tiếp thị.
+• Báo cáo tài chính &amp; Biểu đồ doanh số Realtime qua Recharts; Phân tích phễu chuyển đổi (Traffic -&gt; Click -&gt; Lead -&gt; Order -&gt; Paid).</t>
         </is>
       </c>
       <c r="J6" s="76" t="inlineStr">
         <is>
           <t>⏳ [KẾ HOẠCH DỰ KIẾN]
-• Kiểm thử an toàn thông tin &amp; bảo mật (Pentest, OWASP Top 10, SQLi, XSS, CSRF, Rate Limiting &amp; Brute Force Prevention).
-• Rà soát các tiêu chuẩn mã hóa mật khẩu và token.</t>
+• Kiểm thử tích hợp hệ thống toàn diện E2E (End-to-End Testing) bao phủ toàn bộ các quy trình nghiệp vụ và luồng dữ liệu của hệ thống.
+• Kiểm tra ma trận kết nối luồng dữ liệu 4 thành viên (Khách hàng ↔ Shop ↔ KOL ↔ Admin) qua Postman/Newman automation test.</t>
         </is>
       </c>
       <c r="K6" s="76" t="inlineStr">
         <is>
           <t>⏳ [KẾ HOẠCH DỰ KIẾN]
-• Triển khai thử nghiệm UAT (User Acceptance Testing) với người dùng thật (KOL và Chủ gian hàng đối tác D2C Sora Skin).
-• Ghi nhận phản hồi trải nghiệm thực tế.</t>
+• Kiểm thử an toàn thông tin &amp; bảo mật (Pentest, OWASP Top 10, SQLi, XSS, CSRF, Rate Limiting &amp; Brute Force Prevention).
+• Rà soát an ninh chuỗi mã băm SHA-256 Audit Logs, cơ chế mã hóa Argon2id và xác thực 2 lớp OTP Email.</t>
         </is>
       </c>
       <c r="L6" s="76" t="inlineStr">
         <is>
           <t>⏳ [KẾ HOẠCH DỰ KIẾN]
-• Kiểm thử tải trọng và hiệu năng (Load Testing k6/Artillery 1.000 req/s).
-• Tối ưu hóa Database Indexing và cơ chế đệm Redis Caching.</t>
+• Triển khai thử nghiệm UAT (User Acceptance Testing) với người dùng thật (KOL và Chủ shop đối tác D2C Sora Skin).
+• Thu thập ý kiến đánh giá trải nghiệm thực tế về luồng mua hàng, thẩm định đổi trả và xin mẫu thử.</t>
         </is>
       </c>
       <c r="M6" s="76" t="inlineStr">
         <is>
           <t>⏳ [KẾ HOẠCH DỰ KIẾN]
-• Hoàn thiện các điều chỉnh phản hồi sau UAT.
-• Soạn thảo Hướng dẫn sử dụng chi tiết (User Manual) cho 5 vai trò.</t>
+• Kiểm thử tải trọng và hiệu năng cao (Load Testing k6 / Artillery đạt 1.000 req/s).
+• Tối ưu hóa Database Indexing các bảng Orders, Commissions; tinh chỉnh cơ chế đệm Redis Caching.</t>
         </is>
       </c>
       <c r="N6" s="76" t="inlineStr">
         <is>
           <t>⏳ [KẾ HOẠCH DỰ KIẾN]
-• Hoàn thiện toàn văn Báo cáo Đồ án Khóa luận Tốt nghiệp (Final Capstone Thesis Report) theo quy chuẩn FPT University.</t>
+• Hoàn thiện các điều chỉnh phản hồi sau UAT; khắc phục triệt để các lỗi giao diện và trải nghiệm.
+• Soạn thảo tài liệu Hướng dẫn sử dụng chi tiết (User Manual) chuẩn hóa cho 4 vai trò (Admin, Shop, KOL, Khách hàng).</t>
         </is>
       </c>
       <c r="O6" s="76" t="inlineStr">
         <is>
           <t>⏳ [KẾ HOẠCH DỰ KIẾN]
-• Quay video demo kịch bản nghiệp vụ E2E hoàn chỉnh.
-• Đóng gói Docker Compose và triển khai thử nghiệm trên Production Cloud (Render/AWS).</t>
+• Hoàn thiện toàn văn Báo cáo Đồ án Khóa luận Tốt nghiệp (Final Capstone Thesis Report) theo quy chuẩn FPT University.
+• Hoàn thiện phụ lục kỹ thuật, tài liệu thiết kế kiến trúc và nhật ký đóng góp mã nguồn của từng thành viên.</t>
         </is>
       </c>
       <c r="P6" s="76" t="inlineStr">
         <is>
           <t>⏳ [KẾ HOẠCH DỰ KIẾN]
-• Phê duyệt bảo vệ khóa luận: supervisor đề nghị, CNBM xem xét và phê duyệt.
-• Thẩm định danh sách thành viên đủ điều kiện bảo vệ.</t>
+• Quay video demo kịch bản nghiệp vụ E2E hoàn chỉnh; đóng gói Docker Compose và triển khai thử nghiệm trên Production Cloud (Render/AWS).
+• Phê duyệt bảo vệ khóa luận: Supervisor đề nghị, Chủ nhiệm Bộ môn (CNBM) xem xét và phê duyệt danh sách bảo vệ.</t>
         </is>
       </c>
       <c r="Q6" s="76" t="inlineStr">
         <is>
           <t>⏳ [KẾ HOẠCH DỰ KIẾN]
-• Chuẩn bị Slide thuyết trình bảo vệ trước Hội đồng.
-• Diễn tập bảo vệ khóa luận (Mock Defense) &amp; Tiếp thu góp ý của GVHD.</t>
+• Chuẩn bị Slide thuyết trình bảo vệ trước Hội đồng chấm thi Capstone.
+• Diễn tập bảo vệ khóa luận (Mock Defense), tiếp thu góp ý của GVHD &amp; Bảo vệ chính thức trước Hội đồng chấm thi.</t>
         </is>
       </c>
       <c r="R6" s="77" t="n"/>
@@ -8346,25 +8357,25 @@
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="15" customWidth="1" style="45" min="1" max="1"/>
-    <col width="24" customWidth="1" style="45" min="2" max="2"/>
-    <col width="28" customWidth="1" style="45" min="3" max="6"/>
-    <col width="28" customWidth="1" style="45" min="4" max="4"/>
-    <col width="28" customWidth="1" style="45" min="5" max="5"/>
-    <col width="28" customWidth="1" style="45" min="6" max="6"/>
+    <col width="25" customWidth="1" style="45" min="2" max="2"/>
+    <col width="30" customWidth="1" style="45" min="3" max="6"/>
+    <col width="30" customWidth="1" style="45" min="4" max="4"/>
+    <col width="30" customWidth="1" style="45" min="5" max="5"/>
+    <col width="30" customWidth="1" style="45" min="6" max="6"/>
     <col width="32" customWidth="1" style="45" min="7" max="15"/>
     <col width="32" customWidth="1" style="45" min="8" max="8"/>
-    <col width="38" customWidth="1" style="45" min="9" max="9"/>
-    <col width="28" customWidth="1" style="45" min="10" max="10"/>
-    <col width="28" customWidth="1" style="45" min="11" max="11"/>
-    <col width="28" customWidth="1" style="45" min="12" max="12"/>
-    <col width="28" customWidth="1" style="45" min="13" max="13"/>
-    <col width="28" customWidth="1" style="45" min="14" max="14"/>
-    <col width="28" customWidth="1" style="45" min="15" max="15"/>
-    <col width="28" customWidth="1" style="45" min="16" max="20"/>
-    <col width="28" customWidth="1" style="45" min="17" max="17"/>
-    <col width="28" customWidth="1" style="45" min="18" max="18"/>
-    <col width="28" customWidth="1" style="45" min="19" max="19"/>
-    <col width="28" customWidth="1" style="45" min="20" max="20"/>
+    <col width="36" customWidth="1" style="45" min="9" max="9"/>
+    <col width="44" customWidth="1" style="45" min="10" max="10"/>
+    <col width="30" customWidth="1" style="45" min="11" max="11"/>
+    <col width="30" customWidth="1" style="45" min="12" max="12"/>
+    <col width="30" customWidth="1" style="45" min="13" max="13"/>
+    <col width="30" customWidth="1" style="45" min="14" max="14"/>
+    <col width="30" customWidth="1" style="45" min="15" max="15"/>
+    <col width="30" customWidth="1" style="45" min="16" max="20"/>
+    <col width="30" customWidth="1" style="45" min="17" max="17"/>
+    <col width="30" customWidth="1" style="45" min="18" max="18"/>
+    <col width="30" customWidth="1" style="45" min="19" max="19"/>
+    <col width="30" customWidth="1" style="45" min="20" max="20"/>
     <col width="8.77734375" customWidth="1" style="45" min="21" max="27"/>
   </cols>
   <sheetData>
@@ -8621,7 +8632,7 @@
       <c r="Z5" s="19" t="n"/>
       <c r="AA5" s="20" t="n"/>
     </row>
-    <row r="6" ht="140" customHeight="1" s="45">
+    <row r="6" ht="190" customHeight="1" s="45">
       <c r="A6" s="84" t="inlineStr">
         <is>
           <t>SE184251</t>
@@ -8634,92 +8645,92 @@
       </c>
       <c r="C6" s="86" t="inlineStr">
         <is>
-          <t>Kiến trúc SAD, CSDL 21 bảng 3NF, Base Monorepo NestJS + React Vite</t>
+          <t>Kiến trúc hệ thống SAD, Monorepo NestJS+React, CSDL 41 bảng 3NF; Khóa bắt buộc 100% Đăng nhập (loại bỏ hoàn toàn khách vãng lai, Google 1-Click 1.5s)</t>
         </is>
       </c>
       <c r="D6" s="86" t="inlineStr">
         <is>
-          <t>Phân hệ IAM đa vai trò (Argon2id, JWT, 2FA OTP, Google Auth, RBAC)</t>
+          <t>Phân hệ IAM an ninh cao: Quên mật khẩu qua mã OTP Email 5 phút, mã hóa Argon2id &amp; JWT, xác minh mật khẩu khi đổi SĐT/Email giao hàng</t>
         </is>
       </c>
       <c r="E6" s="86" t="inlineStr">
         <is>
-          <t>Quản lý Gian hàng, Sản phẩm, Biến thể &amp; Phân tách SYSTEM_MANAGER vs ADMIN</t>
+          <t>Quỹ bảo chứng Escrow 14 ngày thích ứng nghỉ Lễ/Tết Việt Nam (Adaptive Holiday-Aware Escrow Engine), quyết toán ví CTV 0đ phí ngân hàng (Sổ cái kép)</t>
         </is>
       </c>
       <c r="F6" s="86" t="inlineStr">
         <is>
-          <t>Nghiệp vụ Escrow 14 ngày, Quyết toán ví CTV 0đ phí NH, Tái thiết kế UI Vàng Be</t>
+          <t>Cổng phân xử Trọng tài Khiếu nại Đổi trả độc lập (Admin Split-View), Trung tâm Thông báo toàn sàn thời gian thực &amp; AI Fraud Sentinel chống tự mua</t>
         </is>
       </c>
       <c r="G6" s="87" t="inlineStr">
         <is>
-          <t>✅ Hoàn thành 100% đề cương, kiến trúc CSDL 21 bảng, Base monorepo, Docker Compose.</t>
+          <t>✅ Hoàn thành 100% đề cương, kiến trúc CSDL 41 bảng 3NF, Base monorepo NestJS + React Vite, cấu hình Docker Compose multi-container.</t>
         </is>
       </c>
       <c r="H6" s="87" t="inlineStr">
         <is>
-          <t>✅ Hoàn thành 100% FR-01 → FR-08 (IAM, Quản trị Store, Danh mục Sản phẩm &amp; Media Hub).</t>
+          <t>✅ Hoàn thành phân hệ Xác thực &amp; Phân quyền đa vai trò, bảo mật mật khẩu Argon2id, mã JWT, mã 2FA OTP, Quản trị Store &amp; Sản phẩm, Kho tài nguyên Media Hub.</t>
         </is>
       </c>
-      <c r="I6" s="88" t="inlineStr">
+      <c r="I6" s="87" t="inlineStr">
         <is>
-          <t>⭐ Hoàn thành 100% phân tách SYSTEM_MANAGER vs ADMIN, Tái thiết kế LoginPage Vàng Be, Escrow 14 ngày &amp; Quyết toán ví CTV, Merge origin/main 0 conflict, Build FE (1.01s) &amp; BE 100% không lỗi.</t>
+          <t>✅ Hoàn thành nền tảng Escrow 14 ngày, quyết toán ví CTV 0đ phí ngân hàng, phân tách vai trò SYSTEM_MANAGER vs SYSTEM_ADMIN, Design System Vàng Be.</t>
         </is>
       </c>
-      <c r="J6" s="89" t="inlineStr">
+      <c r="J6" s="88" t="inlineStr">
         <is>
-          <t>⏳ Socket.io Chat realtime đa kênh KOL ⇄ Shop &amp; Động cơ AI Gợi ý KOL.</t>
+          <t>⭐ Hoàn thành 100%: Khóa 100% login (Google 1-Click); Quên MK OTP Email + Argon2id; Quỹ Escrow 14 ngày thích ứng Lễ/Tết; Cổng Trọng tài phân xử khiếu nại (Split-View); Chuông báo realtime; AI Fraud Sentinel; Chuẩn bị kịch bản demo và slide báo cáo Review.</t>
         </is>
       </c>
       <c r="K6" s="89" t="inlineStr">
         <is>
-          <t>⏳ Bảng vinh danh Leaderboard Gamification &amp; Doanh số Realtime qua Recharts.</t>
+          <t>⏳ Tích hợp thông báo đẩy Socket.io cho trung tâm thông báo; Hỗ trợ các thành viên kết nối cổng Chat realtime Khách ⇄ Shop và KOL ⇄ Shop.</t>
         </is>
       </c>
       <c r="L6" s="89" t="inlineStr">
         <is>
-          <t>⏳ Kiểm thử tích hợp E2E toàn diện 32 FRs qua Postman/Newman.</t>
+          <t>⏳ Xây dựng API và giao diện biểu đồ doanh số tài chính Recharts realtime; Kết nối bảng vinh danh Top KOL Leaderboard.</t>
         </is>
       </c>
       <c r="M6" s="89" t="inlineStr">
         <is>
-          <t>⏳ Kiểm thử bảo mật Pentest, OWASP Top 10, SQLi, XSS, CSRF, Rate Limiting.</t>
+          <t>⏳ Xây dựng bộ kịch bản kiểm thử tích hợp E2E tự động qua Newman/Postman; Kiểm tra ma trận luồng dữ liệu 4 thành viên.</t>
         </is>
       </c>
       <c r="N6" s="89" t="inlineStr">
         <is>
-          <t>⏳ Triển khai UAT với KOL và Shop đối tác Sora Skin thực tế.</t>
+          <t>⏳ Thực hiện Pentest an toàn thông tin hệ thống (OWASP Top 10, SQLi, CSRF, Rate Limiting, Brute Force); Rà soát mã hóa Argon2id và Audit Logs.</t>
         </is>
       </c>
       <c r="O6" s="89" t="inlineStr">
         <is>
-          <t>⏳ Kiểm thử tải trọng k6 1.000 req/s, tối ưu Indexing DB &amp; Redis Caching.</t>
+          <t>⏳ Tổ chức buổi thử nghiệm UAT với người dùng thật (KOL và Chủ shop Sora Skin thực tế); Thu thập phản hồi về luồng Escrow và phân xử.</t>
         </is>
       </c>
       <c r="P6" s="89" t="inlineStr">
         <is>
-          <t>⏳ Hoàn thiện phản hồi UAT &amp; Soạn thảo User Manual 5 vai trò.</t>
+          <t>⏳ Thiết lập kịch bản Load Testing k6 1.000 req/s; Tinh chỉnh hiệu năng truy vấn PostgreSQL và Redis Caching.</t>
         </is>
       </c>
       <c r="Q6" s="89" t="inlineStr">
         <is>
-          <t>⏳ Viết toàn văn Báo cáo Đồ án Khóa luận Tốt nghiệp.</t>
+          <t>⏳ Xử lý các vấn đề phát sinh sau UAT; Soạn thảo User Manual phân hệ System Admin &amp; Bảo mật tài chính.</t>
         </is>
       </c>
       <c r="R6" s="89" t="inlineStr">
         <is>
-          <t>⏳ Quay video demo E2E hoàn chỉnh &amp; Đóng gói Docker Production.</t>
+          <t>⏳ Tổng hợp toàn văn Báo cáo Đồ án Tốt nghiệp (Final Capstone Thesis Report) và hoàn thiện các sơ đồ kiến trúc chuẩn.</t>
         </is>
       </c>
       <c r="S6" s="89" t="inlineStr">
         <is>
-          <t>⏳ Supervisor đề nghị &amp; Phê duyệt bảo vệ khóa luận.</t>
+          <t>⏳ Đóng gói Docker Compose Production (Render/AWS); Quay video demo hoàn chỉnh; Hoàn thiện hồ sơ đề nghị bảo vệ khóa luận.</t>
         </is>
       </c>
       <c r="T6" s="89" t="inlineStr">
         <is>
-          <t>⏳ Diễn tập Mock Defense &amp; Bảo vệ chính thức trước Hội đồng.</t>
+          <t>⏳ Soạn thảo Slide thuyết trình bảo vệ; Diễn tập Mock Defense cùng GVHD &amp; Trình bày chính thức trước Hội đồng chấm thi.</t>
         </is>
       </c>
       <c r="U6" s="28" t="n"/>
@@ -8730,7 +8741,7 @@
       <c r="Z6" s="28" t="n"/>
       <c r="AA6" s="28" t="n"/>
     </row>
-    <row r="7" ht="140" customHeight="1" s="45">
+    <row r="7" ht="190" customHeight="1" s="45">
       <c r="A7" s="84" t="inlineStr">
         <is>
           <t>SE180104</t>
@@ -8738,97 +8749,97 @@
       </c>
       <c r="B7" s="85" t="inlineStr">
         <is>
-          <t>Nguyễn Đình Tuấn</t>
+          <t>Nguyễn Phú Quý</t>
         </is>
       </c>
       <c r="C7" s="86" t="inlineStr">
         <is>
-          <t>Động cơ Tracking Smart Link &amp; Dynamic QR Code canvas 512x512</t>
+          <t>Quản lý tồn kho tức thời (Stock Deduction khi chốt đơn), cảnh báo tồn kho thấp (&lt;= 5 sản phẩm), tự khóa nút mua khi hết hàng</t>
         </is>
       </c>
       <c r="D7" s="86" t="inlineStr">
         <is>
-          <t>Cơ chế phân bổ Last-Click Attribution &amp; Lưu cookie tiếp thị 30 ngày</t>
+          <t>Nút cho phép Shop chủ động hủy đơn có chọn lý do -&gt; Tự động hoàn tiền vào ví khách &amp; hủy hoa hồng tạm giữ</t>
         </is>
       </c>
       <c r="E7" s="86" t="inlineStr">
         <is>
-          <t>Thuật toán Redis Sliding Window Rate Limit chống gian lận click spam/bot</t>
+          <t>Shipping Simulator: Tự sinh mã vận đơn chuẩn TMĐT (GHN-XXXXX), in phiếu giao hàng A6 chuẩn có mã vạch Barcode</t>
         </is>
       </c>
       <c r="F7" s="86" t="inlineStr">
         <is>
-          <t>Giao diện Sàn Shopee-style, Search Zoom Modal &amp; Sơ đồ Use Case Bill OTP</t>
+          <t>Màn hình Shop tiếp nhận và thẩm định video mở hộp đổi trả 14 ngày của khách; Quản lý &amp; phát hành Voucher riêng của từng gian hàng</t>
         </is>
       </c>
       <c r="G7" s="87" t="inlineStr">
         <is>
-          <t>✅ Nghiên cứu thuật toán Last-Click 30 ngày và thư viện tạo mã QR Canvas.</t>
+          <t>✅ Nghiên cứu quy trình quản lý kho hàng và cơ chế trừ tồn kho chống bán vượt (Over-selling) trên các sàn TMĐT lớn.</t>
         </is>
       </c>
       <c r="H7" s="87" t="inlineStr">
         <is>
-          <t>✅ Hoàn thành FR-09 → FR-14 (Tracking link, QR Code PNG, Coupon engine, Redis Rate Limit).</t>
+          <t>✅ Xây dựng màn hình danh sách đơn hàng phía Shop và cấu hình các trường trạng thái đơn hàng (PENDING, PROCESSING, SHIPPED).</t>
         </is>
       </c>
-      <c r="I7" s="88" t="inlineStr">
+      <c r="I7" s="87" t="inlineStr">
         <is>
-          <t>⭐ Hoàn thành tích hợp sơ đồ Use Case Bill OTP (drawio), Search Zoom modal và Header công khai (PR #50, #51).</t>
+          <t>✅ Hoàn thiện giao diện hiển thị doanh số Shop phân tách: Doanh thu đang bảo chứng Escrow vs Doanh thu khả dụng.</t>
         </is>
       </c>
-      <c r="J7" s="89" t="inlineStr">
+      <c r="J7" s="88" t="inlineStr">
         <is>
-          <t>⏳ Tối ưu giao diện tạo link tiếp thị nhanh từ extension/bookmarklet.</t>
+          <t>⭐ Hoàn thành: Trừ kho tức thời &amp; cảnh báo tồn kho &lt;= 5; Nút Shop hủy đơn kèm hoàn tiền tự động; Shipping Simulator in phiếu A6 Barcode; Thẩm định video đổi trả 14 ngày; Voucher riêng của shop; Sẵn sàng kịch bản demo Review.</t>
         </is>
       </c>
       <c r="K7" s="89" t="inlineStr">
         <is>
-          <t>⏳ Biểu đồ phân tích lượt click và tỷ lệ chuyển đổi theo kênh MXH.</t>
+          <t>⏳ Tối ưu giao diện in phiếu vận đơn A6 tương thích nhiều khổ máy in nhiệt; Kết nối module Chat Shop ⇄ Khách từ chi tiết đơn hàng.</t>
         </is>
       </c>
       <c r="L7" s="89" t="inlineStr">
         <is>
-          <t>⏳ Kiểm thử E2E luồng quét QR -&gt; Ghi nhận cookie -&gt; Tạo đơn hàng.</t>
+          <t>⏳ Biểu đồ phân tích doanh thu và số lượng đơn hàng theo từng sản phẩm của Shop trên Dashboard.</t>
         </is>
       </c>
       <c r="M7" s="89" t="inlineStr">
         <is>
-          <t>⏳ Thử nghiệm tấn công brute-force click traffic để kiểm tra Redis Rate Limit.</t>
+          <t>⏳ Kiểm thử E2E luồng: Khách đặt hàng -&gt; Trừ kho -&gt; Shop in phiếu giao -&gt; Shipping Simulator -&gt; Hoàn tất đơn.</t>
         </is>
       </c>
       <c r="N7" s="89" t="inlineStr">
         <is>
-          <t>⏳ Hỗ trợ người dùng UAT thử nghiệm tính năng tạo link và quét mã QR.</t>
+          <t>⏳ Kiểm thử an ninh luồng hủy đơn hàng và hoàn tiền, đảm bảo không bị lỗi race-condition hoặc âm tiền quỹ.</t>
         </is>
       </c>
       <c r="O7" s="89" t="inlineStr">
         <is>
-          <t>⏳ Tối ưu hóa tốc độ redirect link rút gọn qua Redis cache &lt; 50ms.</t>
+          <t>⏳ Hỗ trợ Chủ shop Sora Skin chạy thử tính năng quản lý kho, in vận đơn A6 và tiếp nhận thẩm định đổi trả trong đợt UAT.</t>
         </is>
       </c>
       <c r="P7" s="89" t="inlineStr">
         <is>
-          <t>⏳ Soạn thảo tài liệu hướng dẫn tạo link và QR cho KOL.</t>
+          <t>⏳ Tối ưu hóa truy vấn Database danh sách đơn hàng và tồn kho sản phẩm khi lượng đơn phát sinh lớn.</t>
         </is>
       </c>
       <c r="Q7" s="89" t="inlineStr">
         <is>
-          <t>⏳ Viết phần Báo cáo Đồ án về Phân hệ Tracking Tiếp thị.</t>
+          <t>⏳ Soạn thảo tài liệu hướng dẫn sử dụng (User Manual) dành riêng cho vai trò Merchant (Chủ gian hàng).</t>
         </is>
       </c>
       <c r="R7" s="89" t="inlineStr">
         <is>
-          <t>⏳ Chuẩn bị kịch bản demo tính năng quét QR và tracking chuyển đổi.</t>
+          <t>⏳ Viết phần Báo cáo Đồ án về Phân hệ Quản Trị Gian Hàng, Vận Chuyển và Xử Lý Đơn Hàng.</t>
         </is>
       </c>
       <c r="S7" s="89" t="inlineStr">
         <is>
-          <t>⏳ Hoàn thiện hồ sơ nghiệm thu kỹ thuật phân hệ Tracking.</t>
+          <t>⏳ Chuẩn bị kịch bản demo tính năng Quản lý kho, In phiếu A6 Barcode và Thẩm định video đổi trả.</t>
         </is>
       </c>
       <c r="T7" s="89" t="inlineStr">
         <is>
-          <t>⏳ Trình bày slide phần Tracking &amp; QR Code trước Hội đồng.</t>
+          <t>⏳ Trình bày slide phần Quản Trị Gian Hàng &amp; Vận Chuyển trước Hội đồng chấm thi.</t>
         </is>
       </c>
       <c r="U7" s="28" t="n"/>
@@ -8839,7 +8850,7 @@
       <c r="Z7" s="28" t="n"/>
       <c r="AA7" s="28" t="n"/>
     </row>
-    <row r="8" ht="140" customHeight="1" s="45">
+    <row r="8" ht="190" customHeight="1" s="45">
       <c r="A8" s="84" t="inlineStr">
         <is>
           <t>SE180104</t>
@@ -8847,97 +8858,97 @@
       </c>
       <c r="B8" s="85" t="inlineStr">
         <is>
-          <t>Nguyễn Phú Quý</t>
+          <t>Nguyễn Đình Tuấn</t>
         </is>
       </c>
       <c r="C8" s="86" t="inlineStr">
         <is>
-          <t>Động cơ AI Fraud Sentinel phát hiện gian lận traffic bất thường</t>
+          <t>Cơ chế phân cấp hoa hồng tiếp thị 2 tầng: Mức cơ bản (Open Offer) tự lấy link vs Mức độc quyền (Exclusive Deal) đàm phán qua Chat</t>
         </is>
       </c>
       <c r="D8" s="86" t="inlineStr">
         <is>
-          <t>Chuỗi an ninh kiểm toán Audit Logs bất biến (mã băm SHA-256)</t>
+          <t>Quy trình yêu cầu cấp sản phẩm mẫu 4 bước (Sample Request Flow) có cam kết trả video review trong vòng 14 ngày</t>
         </is>
       </c>
       <c r="E8" s="86" t="inlineStr">
         <is>
-          <t>Trợ lý AI Gợi ý KOL phù hợp với danh mục sản phẩm (Recommendation)</t>
+          <t>Hệ thống Voucher Livestream theo phiên phát sóng với đồng hồ đếm ngược (Countdown Timer) tự hủy khi hết live</t>
         </is>
       </c>
       <c r="F8" s="86" t="inlineStr">
         <is>
-          <t>Xây dựng và kiểm thử 16/16 Integration &amp; E2E Test suites an ninh mạng</t>
+          <t>Hàng đợi Admin kiểm duyệt hồ sơ Shop mới (KYC CCCD, MST, ĐKKD, STK) &amp; Kiểm duyệt nội dung sản phẩm mới (DRAFT -&gt; APPROVED)</t>
         </is>
       </c>
       <c r="G8" s="87" t="inlineStr">
         <is>
-          <t>✅ Nghiên cứu mô hình phát hiện gian lận traffic (IP spoofing, bot traffic).</t>
+          <t>✅ Nghiên cứu quy chế kiểm duyệt thông tin nhãn hàng và thuật toán phân bổ hoa hồng đa tầng của TikTok Shop Creator.</t>
         </is>
       </c>
       <c r="H8" s="87" t="inlineStr">
         <is>
-          <t>✅ Hoàn thành FR-31 (AI Fraud Sentinel) &amp; FR-32 (Audit Logs) kèm 16/16 E2E test suites (PR #41).</t>
+          <t>✅ Hoàn thành động cơ tạo link tiếp thị rút gọn, Dynamic QR Code canvas 512x512, cookie lưu trữ 30 ngày và thuật toán ngăn chặn click ảo.</t>
         </is>
       </c>
-      <c r="I8" s="88" t="inlineStr">
+      <c r="I8" s="87" t="inlineStr">
         <is>
-          <t>⭐ Duy trì kiểm thử bảo mật cho luồng phân tách SYSTEM_MANAGER, rà soát nhật ký audit log cho luồng phê duyệt KYC.</t>
+          <t>✅ Hoàn thành tích hợp sơ đồ Use Case Bill OTP (drawio), Search Zoom modal và Header công khai (PR #50, #51).</t>
         </is>
       </c>
-      <c r="J8" s="89" t="inlineStr">
+      <c r="J8" s="88" t="inlineStr">
         <is>
-          <t>⏳ Huấn luyện thuật toán AI Recommendation gợi ý KOL theo độ tương đồng sản phẩm.</t>
+          <t>⭐ Hoàn thành: Hoa hồng 2 tầng (Open Offer vs Deal riêng); Quy trình xin mẫu thử 4 bước; Voucher Live đếm ngược tự hủy; Hàng đợi duyệt Shop &amp; Sản phẩm mới; Sẵn sàng dữ liệu demo Review.</t>
         </is>
       </c>
       <c r="K8" s="89" t="inlineStr">
         <is>
-          <t>⏳ Bảng cảnh báo rủi ro gian lận Realtime trên Dashboard Admin.</t>
+          <t>⏳ Tích hợp đồng hồ đếm ngược Voucher Live vào phòng Livestream; Xây dựng màn hình đàm phán Exclusive Deal trực tiếp qua Chat.</t>
         </is>
       </c>
       <c r="L8" s="89" t="inlineStr">
         <is>
-          <t>⏳ Viết kịch bản kiểm thử tự động cho động cơ AI Fraud Sentinel.</t>
+          <t>⏳ Biểu đồ theo dõi tỷ lệ chuyển đổi đơn hàng và hiệu quả doanh số của từng mã tracking link KOL.</t>
         </is>
       </c>
       <c r="M8" s="89" t="inlineStr">
         <is>
-          <t>⏳ Rà soát an ninh chuỗi khối hash SHA-256 chống giả mạo nhật ký giao dịch.</t>
+          <t>⏳ Kiểm thử E2E luồng: KOL xin mẫu thử -&gt; Shop duyệt gửi -&gt; KOL nhận mẫu nộp video -&gt; Lấy link tiếp thị bán hàng.</t>
         </is>
       </c>
       <c r="N8" s="89" t="inlineStr">
         <is>
-          <t>⏳ Thu thập đánh giá từ Admin và Shop về độ chính xác của AI Recommendation.</t>
+          <t>⏳ Kiểm thử an toàn luồng duyệt hồ sơ KYC và cơ chế tự khóa tài khoản KOL khi quá hạn 14 ngày không nộp video review.</t>
         </is>
       </c>
       <c r="O8" s="89" t="inlineStr">
         <is>
-          <t>⏳ Tối ưu hóa thời gian phản hồi của mô hình AI &lt; 200ms.</t>
+          <t>⏳ Hỗ trợ các bạn KOL chạy thử tính năng xin hàng mẫu, lấy link tiếp thị và áp voucher phiên livestream trong đợt UAT.</t>
         </is>
       </c>
       <c r="P8" s="89" t="inlineStr">
         <is>
-          <t>⏳ Hoàn thiện tài liệu kiến trúc AI Sentinel và Audit Logs.</t>
+          <t>⏳ Tối ưu hóa hiệu năng hàng đợi kiểm duyệt KYC và tốc độ truy vấn kho hàng tiếp thị của KOL.</t>
         </is>
       </c>
       <c r="Q8" s="89" t="inlineStr">
         <is>
-          <t>⏳ Viết phần Báo cáo Đồ án về Ứng dụng Trí tuệ Nhân tạo &amp; Bảo mật Audit Trail.</t>
+          <t>⏳ Soạn thảo tài liệu hướng dẫn sử dụng (User Manual) dành cho KOL/KOC và Quản trị viên kiểm duyệt.</t>
         </is>
       </c>
       <c r="R8" s="89" t="inlineStr">
         <is>
-          <t>⏳ Demo kịch bản phát hiện và ngăn chặn gian lận traffic thời gian thực.</t>
+          <t>⏳ Viết phần Báo cáo Đồ án về Phân hệ Tiếp Thị Liên Kết KOL/KOC và Quy Trình Kiểm Duyệt Sàn.</t>
         </is>
       </c>
       <c r="S8" s="89" t="inlineStr">
         <is>
-          <t>⏳ Đóng gói mô hình AI và tài liệu nghiệm thu bảo mật.</t>
+          <t>⏳ Chuẩn bị kịch bản demo luồng Xin mẫu thử 4 bước, Hoa hồng 2 tầng và Voucher phiên live đếm ngược.</t>
         </is>
       </c>
       <c r="T8" s="89" t="inlineStr">
         <is>
-          <t>⏳ Trình bày slide giải pháp AI và Bảo mật trước Hội đồng.</t>
+          <t>⏳ Trình bày slide phần Mạng Lưới KOL &amp; Kiểm Duyệt Sàn trước Hội đồng chấm thi.</t>
         </is>
       </c>
       <c r="U8" s="28" t="n"/>
@@ -8948,7 +8959,7 @@
       <c r="Z8" s="28" t="n"/>
       <c r="AA8" s="28" t="n"/>
     </row>
-    <row r="9" ht="140" customHeight="1" s="45">
+    <row r="9" ht="190" customHeight="1" s="45">
       <c r="A9" s="84" t="inlineStr">
         <is>
           <t>SE184527</t>
@@ -8961,92 +8972,92 @@
       </c>
       <c r="C9" s="86" t="inlineStr">
         <is>
-          <t>Giỏ hàng đồng bộ Database PostgreSQL, lưu trữ tập trung</t>
+          <t>Giỏ hàng đồng bộ Database PostgreSQL, lưu trữ tập trung, đồng bộ tức thời đa thiết bị (Omnichannel Cart Persistence)</t>
         </is>
       </c>
       <c r="D9" s="86" t="inlineStr">
         <is>
-          <t>Quy trình gửi yêu cầu Đổi trả 14 ngày (bắt buộc video mở hộp)</t>
+          <t>Quy trình gửi yêu cầu Đổi trả / Hoàn tiền 14 ngày (bắt buộc đính kèm ảnh và video mở hộp chống tráo hàng)</t>
         </is>
       </c>
       <c r="E9" s="86" t="inlineStr">
         <is>
-          <t>Ràng buộc đánh giá thật (Review Gate: đơn COMPLETED mới được review)</t>
+          <t>Ràng buộc đánh giá thật (Verified Review Gate: Chỉ đơn hàng COMPLETED mới được mở quyền review 5 sao)</t>
         </is>
       </c>
       <c r="F9" s="86" t="inlineStr">
         <is>
-          <t>Trang chính sách gian hàng trước checkout &amp; Chat Khách ⇄ Shop</t>
+          <t>Minh bạch chính sách bảo hành gian hàng trước checkout &amp; Kênh chat tư vấn trực tiếp Khách hàng ⇄ Chủ Shop (Live In-App Chat)</t>
         </is>
       </c>
       <c r="G9" s="87" t="inlineStr">
         <is>
-          <t>✅ Nghiên cứu cơ chế giỏ hàng đồng bộ đa thiết bị và quy định đổi trả E-commerce.</t>
+          <t>✅ Nghiên cứu cơ chế đồng bộ giỏ hàng qua Database PostgreSQL và Luật Bảo vệ quyền lợi người tiêu dùng trong mua sắm online.</t>
         </is>
       </c>
       <c r="H9" s="87" t="inlineStr">
         <is>
-          <t>✅ Hoàn thành cấu hình Cổng Khách Hàng (Customer Portal) và sổ địa chỉ giao hàng.</t>
+          <t>✅ Hoàn thành cấu hình Cổng Khách Hàng (Customer Portal), quản lý thông tin tài khoản và sổ địa chỉ giao hàng.</t>
         </is>
       </c>
-      <c r="I9" s="88" t="inlineStr">
+      <c r="I9" s="87" t="inlineStr">
         <is>
-          <t>⭐ Hoàn thành luồng Đổi trả 14 ngày phía Khách (đính kèm video), Ràng buộc đánh giá chỉ cho đơn COMPLETED, Giỏ hàng đồng bộ Database.</t>
+          <t>✅ Hoàn thành tích hợp giao diện hiển thị trạng thái đơn hàng phía Khách và liên kết xem hành trình giao nhận.</t>
         </is>
       </c>
-      <c r="J9" s="89" t="inlineStr">
+      <c r="J9" s="88" t="inlineStr">
         <is>
-          <t>⏳ Hoàn thiện giao diện Chat trực tiếp Khách hàng ⇄ Chủ Shop từ trang chi tiết sản phẩm.</t>
+          <t>⭐ Hoàn thành: Giỏ hàng đồng bộ Database PostgreSQL; Khiếu nại đổi trả 14 ngày bắt buộc video mở hộp; Ràng buộc đánh giá thật Verified Review Gate; Chat tư vấn Khách ⇄ Shop; Sẵn sàng kịch bản demo Review.</t>
         </is>
       </c>
       <c r="K9" s="89" t="inlineStr">
         <is>
-          <t>⏳ Tối ưu hóa trải nghiệm xem đơn hàng và tiến độ hoàn tiền trực quan.</t>
+          <t>⏳ Hoàn thiện giao diện Chat trực tiếp Khách hàng ⇄ Chủ Shop thời gian thực; Hiển thị danh thiếp sản phẩm ngay trong khung chat.</t>
         </is>
       </c>
       <c r="L9" s="89" t="inlineStr">
         <is>
-          <t>⏳ Kiểm thử tích hợp E2E luồng: Thêm giỏ -&gt; Đặt hàng -&gt; Nhận hàng -&gt; Đổi trả.</t>
+          <t>⏳ Tối ưu hóa trang 'Đơn mua của tôi' với thanh tiến trình trực quan (Timeline: Đặt hàng -&gt; Đang giao -&gt; Đã giao -&gt; Hoàn tất).</t>
         </is>
       </c>
       <c r="M9" s="89" t="inlineStr">
         <is>
-          <t>⏳ Kiểm thử an toàn thông tin giỏ hàng và dữ liệu địa chỉ khách hàng.</t>
+          <t>⏳ Kiểm thử tích hợp E2E luồng: Thêm giỏ hàng -&gt; Đặt hàng -&gt; Nhận hàng -&gt; Gửi yêu cầu đổi trả có video mở hộp.</t>
         </is>
       </c>
       <c r="N9" s="89" t="inlineStr">
         <is>
-          <t>⏳ Kiểm thử UAT với người dùng thật về trải nghiệm mua sắm và gửi khiếu nại.</t>
+          <t>⏳ Kiểm thử an toàn thông tin dữ liệu khách hàng, chống tấn công thao túng giỏ hàng hoặc gửi đánh giá giả mạo.</t>
         </is>
       </c>
       <c r="O9" s="89" t="inlineStr">
         <is>
-          <t>⏳ Tối ưu hóa truy vấn Database giỏ hàng và danh sách đơn mua của khách.</t>
+          <t>⏳ Theo dõi người dùng thật thử nghiệm trải nghiệm mua sắm, thêm giỏ hàng đa thiết bị và viết đánh giá trong đợt UAT.</t>
         </is>
       </c>
       <c r="P9" s="89" t="inlineStr">
         <is>
-          <t>⏳ Soạn thảo tài liệu hướng dẫn mua sắm và quy trình khiếu nại đổi trả cho khách.</t>
+          <t>⏳ Tối ưu hóa câu truy vấn Database giỏ hàng và danh sách lịch sử đơn mua của khách hàng.</t>
         </is>
       </c>
       <c r="Q9" s="89" t="inlineStr">
         <is>
-          <t>⏳ Viết phần Báo cáo Đồ án về Phân hệ Khách Hàng &amp; Trải Nghiệm Mua Sắm.</t>
+          <t>⏳ Soạn thảo tài liệu hướng dẫn mua sắm và quy trình khiếu nại đổi trả (User Guide) cho Khách mua hàng.</t>
         </is>
       </c>
       <c r="R9" s="89" t="inlineStr">
         <is>
-          <t>⏳ Chuẩn bị kịch bản demo hành trình mua sắm, nhận hàng và đánh giá sản phẩm.</t>
+          <t>⏳ Viết phần Báo cáo Đồ án về Phân hệ Khách Mua Hàng &amp; Trải Nghiệm Mua Sắm E-Commerce.</t>
         </is>
       </c>
       <c r="S9" s="89" t="inlineStr">
         <is>
-          <t>⏳ Hoàn thiện hồ sơ nghiệm thu kỹ thuật phân hệ Khách Hàng.</t>
+          <t>⏳ Chuẩn bị kịch bản demo hành trình khách mua hàng: Giỏ hàng đồng bộ, Đổi trả video mở hộp và Đánh giá Verified Buyer.</t>
         </is>
       </c>
       <c r="T9" s="89" t="inlineStr">
         <is>
-          <t>⏳ Trình bày slide phần Cổng Khách Hàng &amp; Đổi Trả trước Hội đồng.</t>
+          <t>⏳ Trình bày slide phần Cổng Khách Hàng &amp; Trải Nghiệm Mua Sắm trước Hội đồng chấm thi.</t>
         </is>
       </c>
       <c r="U9" s="28" t="n"/>
@@ -15958,8 +15969,8 @@
     <row r="1000" ht="14.25" customHeight="1" s="45"/>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="C4:F4"/>
     <mergeCell ref="G4:T4"/>
-    <mergeCell ref="C4:F4"/>
     <mergeCell ref="A4:A5"/>
     <mergeCell ref="B4:B5"/>
   </mergeCells>

</xml_diff>